<commit_message>
move not use markevalueData
</commit_message>
<xml_diff>
--- a/data/analysis/momentumNew/mergeTtestResult/merged_t_test.xlsx
+++ b/data/analysis/momentumNew/mergeTtestResult/merged_t_test.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\Han\學習\金融策略\分析程式\data\analysis\momentumNew\mergeTtestResult\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56B00524-421A-4D13-AA67-B05EDD2B73A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6557CE94-440C-4568-AE55-19E2F958E748}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{79B926A8-815C-4ADE-A3A1-103001E1D343}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="2" xr2:uid="{79B926A8-815C-4ADE-A3A1-103001E1D343}"/>
   </bookViews>
   <sheets>
     <sheet name="merged_t_test" sheetId="1" r:id="rId1"/>
+    <sheet name="15years" sheetId="2" r:id="rId2"/>
+    <sheet name="improved" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">merged_t_test!$A$1:$G$49</definedName>
@@ -1046,7 +1048,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1106,21 +1108,6 @@
     </xf>
     <xf numFmtId="176" fontId="14" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="21" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1128,6 +1115,87 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="22" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="22" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="21" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="35" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="22" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="22" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="21" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="14" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="22" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="21" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="21" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1143,91 +1211,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="22" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="22" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="21" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="35" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="22" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="22" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="21" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="14" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="22" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="21" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="21" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1602,7 +1586,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{828DFD01-9D50-4EA6-A7DD-A0B766D34BA5}">
-  <dimension ref="A1:N61"/>
+  <dimension ref="A1:N59"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="11.375" style="8" customWidth="1"/>
@@ -1706,14 +1690,14 @@
       <c r="G4" s="9">
         <v>5.1106356269530005E-4</v>
       </c>
-      <c r="I4" s="39" t="s">
+      <c r="I4" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="J4" s="38"/>
-      <c r="K4" s="38"/>
-      <c r="L4" s="38"/>
-      <c r="M4" s="38"/>
-      <c r="N4" s="40"/>
+      <c r="J4" s="47"/>
+      <c r="K4" s="47"/>
+      <c r="L4" s="47"/>
+      <c r="M4" s="47"/>
+      <c r="N4" s="48"/>
     </row>
     <row r="5" spans="1:14" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7">
@@ -1737,10 +1721,10 @@
       <c r="G5" s="10">
         <v>0.25494625406830401</v>
       </c>
-      <c r="I5" s="41" t="s">
+      <c r="I5" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="J5" s="26" t="s">
+      <c r="J5" s="21" t="s">
         <v>45</v>
       </c>
       <c r="K5" s="15">
@@ -1752,7 +1736,7 @@
       <c r="M5" s="15">
         <v>9</v>
       </c>
-      <c r="N5" s="42">
+      <c r="N5" s="29">
         <v>12</v>
       </c>
     </row>
@@ -1778,25 +1762,25 @@
       <c r="G6" s="10">
         <v>7.9232025762956804E-6</v>
       </c>
-      <c r="I6" s="43">
+      <c r="I6" s="54">
         <v>3</v>
       </c>
-      <c r="J6" s="27" t="s">
+      <c r="J6" s="49" t="s">
         <v>7</v>
       </c>
-      <c r="K6" s="21">
+      <c r="K6" s="14">
         <f>$E2</f>
         <v>3.0260421823129999E-4</v>
       </c>
-      <c r="L6" s="21">
+      <c r="L6" s="14">
         <f>$E5</f>
         <v>1.51301049852723E-2</v>
       </c>
-      <c r="M6" s="21">
+      <c r="M6" s="14">
         <f>$E8</f>
         <v>1.51244575442856E-2</v>
       </c>
-      <c r="N6" s="44">
+      <c r="N6" s="30">
         <f>$E11</f>
         <v>2.3280515551955899E-2</v>
       </c>
@@ -1823,21 +1807,21 @@
       <c r="G7" s="10">
         <v>2.184178713642E-4</v>
       </c>
-      <c r="I7" s="45"/>
-      <c r="J7" s="28"/>
-      <c r="K7" s="25" t="str">
+      <c r="I7" s="43"/>
+      <c r="J7" s="50"/>
+      <c r="K7" s="20" t="str">
         <f>"("&amp;TEXT($F2, "0.00")&amp;")"</f>
         <v>(0.03)</v>
       </c>
-      <c r="L7" s="25" t="str">
+      <c r="L7" s="20" t="str">
         <f>"("&amp;TEXT($F5, "0.00")&amp;")"</f>
         <v>(1.14)</v>
       </c>
-      <c r="M7" s="25" t="str">
+      <c r="M7" s="20" t="str">
         <f>"("&amp;TEXT($F8, "0.00")&amp;")"</f>
         <v>(0.96)</v>
       </c>
-      <c r="N7" s="46" t="str">
+      <c r="N7" s="31" t="str">
         <f>"("&amp;TEXT($F11, "0.00")&amp;")"</f>
         <v>(1.16)</v>
       </c>
@@ -1864,23 +1848,23 @@
       <c r="G8" s="9">
         <v>0.34096046080184</v>
       </c>
-      <c r="I8" s="45"/>
-      <c r="J8" s="29" t="s">
+      <c r="I8" s="43"/>
+      <c r="J8" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="K8" s="47">
+      <c r="K8" s="32">
         <f>$E3</f>
         <v>3.0722210317410001E-2</v>
       </c>
-      <c r="L8" s="47">
+      <c r="L8" s="32">
         <f>$E6</f>
         <v>6.5631060309720005E-2</v>
       </c>
-      <c r="M8" s="47">
+      <c r="M8" s="32">
         <f>$E9</f>
         <v>9.0526528336692905E-2</v>
       </c>
-      <c r="N8" s="48">
+      <c r="N8" s="33">
         <f>$E12</f>
         <v>9.33097832882889E-2</v>
       </c>
@@ -1907,21 +1891,21 @@
       <c r="G9" s="9">
         <v>1.2141876138480901E-6</v>
       </c>
-      <c r="I9" s="45"/>
-      <c r="J9" s="28"/>
-      <c r="K9" s="36" t="str">
+      <c r="I9" s="43"/>
+      <c r="J9" s="50"/>
+      <c r="K9" s="26" t="str">
         <f>"("&amp;TEXT($F3,"0.00")&amp;")"</f>
         <v>(3.55)</v>
       </c>
-      <c r="L9" s="36" t="str">
+      <c r="L9" s="26" t="str">
         <f>"("&amp;TEXT($F6,"0.00")&amp;")"</f>
         <v>(4.69)</v>
       </c>
-      <c r="M9" s="36" t="str">
+      <c r="M9" s="26" t="str">
         <f>"("&amp;TEXT($F9,"0.00")&amp;")"</f>
         <v>(5.15)</v>
       </c>
-      <c r="N9" s="49" t="str">
+      <c r="N9" s="34" t="str">
         <f>"("&amp;TEXT($F12,"0.00")&amp;")"</f>
         <v>(4.41)</v>
       </c>
@@ -1948,23 +1932,23 @@
       <c r="G10" s="9">
         <v>1.7724280876774E-5</v>
       </c>
-      <c r="I10" s="45"/>
-      <c r="J10" s="30" t="s">
-        <v>9</v>
-      </c>
-      <c r="K10" s="47">
+      <c r="I10" s="43"/>
+      <c r="J10" s="52" t="s">
+        <v>9</v>
+      </c>
+      <c r="K10" s="32">
         <f>$E4</f>
         <v>3.0419606099178698E-2</v>
       </c>
-      <c r="L10" s="47">
+      <c r="L10" s="32">
         <f>$E7</f>
         <v>5.0500955324447698E-2</v>
       </c>
-      <c r="M10" s="47">
+      <c r="M10" s="32">
         <f>$E10</f>
         <v>7.5402070792407294E-2</v>
       </c>
-      <c r="N10" s="48">
+      <c r="N10" s="33">
         <f>$E13</f>
         <v>7.0029267736333001E-2</v>
       </c>
@@ -1991,21 +1975,21 @@
       <c r="G11" s="10">
         <v>0.24789234222405299</v>
       </c>
-      <c r="I11" s="50"/>
-      <c r="J11" s="31"/>
-      <c r="K11" s="37" t="str">
+      <c r="I11" s="44"/>
+      <c r="J11" s="53"/>
+      <c r="K11" s="27" t="str">
         <f>"("&amp;TEXT($F4,"0.00")&amp;")"</f>
         <v>(3.58)</v>
       </c>
-      <c r="L11" s="37" t="str">
+      <c r="L11" s="27" t="str">
         <f>"("&amp;TEXT($F7,"0.00")&amp;")"</f>
         <v>(3.82)</v>
       </c>
-      <c r="M11" s="37" t="str">
+      <c r="M11" s="27" t="str">
         <f>"("&amp;TEXT($F10,"0.00")&amp;")"</f>
         <v>(4.49)</v>
       </c>
-      <c r="N11" s="51" t="str">
+      <c r="N11" s="35" t="str">
         <f>"("&amp;TEXT($F13,"0.00")&amp;")"</f>
         <v>(3.39)</v>
       </c>
@@ -2032,22 +2016,22 @@
       <c r="G12" s="10">
         <v>2.5034503907783899E-5</v>
       </c>
-      <c r="I12" s="52">
+      <c r="I12" s="42">
         <v>6</v>
       </c>
-      <c r="J12" s="32" t="s">
+      <c r="J12" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="K12" s="21">
+      <c r="K12" s="14">
         <v>4.7735012474096001E-3</v>
       </c>
-      <c r="L12" s="21">
+      <c r="L12" s="14">
         <v>1.89783044088855E-2</v>
       </c>
-      <c r="M12" s="21">
+      <c r="M12" s="14">
         <v>1.99711867006667E-2</v>
       </c>
-      <c r="N12" s="44">
+      <c r="N12" s="30">
         <v>3.0649711185840801E-2</v>
       </c>
     </row>
@@ -2073,18 +2057,18 @@
       <c r="G13" s="10">
         <v>9.8533179837500011E-4</v>
       </c>
-      <c r="I13" s="45"/>
-      <c r="J13" s="33"/>
-      <c r="K13" s="25" t="s">
+      <c r="I13" s="43"/>
+      <c r="J13" s="23"/>
+      <c r="K13" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="L13" s="25" t="s">
+      <c r="L13" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="M13" s="25" t="s">
+      <c r="M13" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="N13" s="46" t="s">
+      <c r="N13" s="31" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2110,20 +2094,20 @@
       <c r="G14" s="9">
         <v>0.65423383389473</v>
       </c>
-      <c r="I14" s="45"/>
-      <c r="J14" s="32" t="s">
+      <c r="I14" s="43"/>
+      <c r="J14" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="K14" s="47">
+      <c r="K14" s="32">
         <v>2.7115683765055399E-2</v>
       </c>
-      <c r="L14" s="47">
+      <c r="L14" s="32">
         <v>5.4315765000363898E-2</v>
       </c>
-      <c r="M14" s="47">
+      <c r="M14" s="32">
         <v>6.03256929965394E-2</v>
       </c>
-      <c r="N14" s="48">
+      <c r="N14" s="33">
         <v>5.3065850483251402E-2</v>
       </c>
     </row>
@@ -2149,18 +2133,18 @@
       <c r="G15" s="9">
         <v>2.1961835765053998E-3</v>
       </c>
-      <c r="I15" s="45"/>
-      <c r="J15" s="33"/>
-      <c r="K15" s="36" t="s">
+      <c r="I15" s="43"/>
+      <c r="J15" s="23"/>
+      <c r="K15" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="L15" s="36" t="s">
+      <c r="L15" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="M15" s="36" t="s">
+      <c r="M15" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="N15" s="49" t="s">
+      <c r="N15" s="34" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2186,20 +2170,20 @@
       <c r="G16" s="9">
         <v>8.3279350537053005E-3</v>
       </c>
-      <c r="I16" s="45"/>
-      <c r="J16" s="34" t="s">
-        <v>9</v>
-      </c>
-      <c r="K16" s="47">
+      <c r="I16" s="43"/>
+      <c r="J16" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="K16" s="32">
         <v>2.23421825176458E-2</v>
       </c>
-      <c r="L16" s="47">
+      <c r="L16" s="32">
         <v>3.5337460591478298E-2</v>
       </c>
-      <c r="M16" s="47">
+      <c r="M16" s="32">
         <v>4.0354506295872603E-2</v>
       </c>
-      <c r="N16" s="44">
+      <c r="N16" s="30">
         <v>2.2416139297410601E-2</v>
       </c>
     </row>
@@ -2225,18 +2209,18 @@
       <c r="G17" s="10">
         <v>0.18067514945157101</v>
       </c>
-      <c r="I17" s="50"/>
-      <c r="J17" s="35"/>
+      <c r="I17" s="44"/>
+      <c r="J17" s="25"/>
       <c r="K17" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="L17" s="37" t="s">
+      <c r="L17" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="M17" s="37" t="s">
+      <c r="M17" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="N17" s="53" t="s">
+      <c r="N17" s="36" t="s">
         <v>27</v>
       </c>
     </row>
@@ -2262,22 +2246,22 @@
       <c r="G18" s="10">
         <v>6.0419980721123302E-5</v>
       </c>
-      <c r="I18" s="52">
-        <v>9</v>
-      </c>
-      <c r="J18" s="32" t="s">
+      <c r="I18" s="42">
+        <v>9</v>
+      </c>
+      <c r="J18" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="K18" s="21">
+      <c r="K18" s="14">
         <v>5.9719290995810005E-4</v>
       </c>
-      <c r="L18" s="21">
+      <c r="L18" s="14">
         <v>6.1873933427599999E-4</v>
       </c>
-      <c r="M18" s="21">
+      <c r="M18" s="14">
         <v>1.523367447362E-3</v>
       </c>
-      <c r="N18" s="44">
+      <c r="N18" s="30">
         <v>1.5399793559194999E-2</v>
       </c>
     </row>
@@ -2303,18 +2287,18 @@
       <c r="G19" s="10">
         <v>3.5367985366198001E-3</v>
       </c>
-      <c r="I19" s="45"/>
-      <c r="J19" s="33"/>
-      <c r="K19" s="25" t="s">
+      <c r="I19" s="43"/>
+      <c r="J19" s="23"/>
+      <c r="K19" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="L19" s="25" t="s">
+      <c r="L19" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="M19" s="25" t="s">
+      <c r="M19" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="N19" s="46" t="s">
+      <c r="N19" s="31" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2340,20 +2324,20 @@
       <c r="G20" s="9">
         <v>0.231100321207518</v>
       </c>
-      <c r="I20" s="45"/>
-      <c r="J20" s="32" t="s">
+      <c r="I20" s="43"/>
+      <c r="J20" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="K20" s="47">
+      <c r="K20" s="32">
         <v>2.8474975298435901E-2</v>
       </c>
-      <c r="L20" s="47">
+      <c r="L20" s="32">
         <v>4.1623593254200397E-2</v>
       </c>
-      <c r="M20" s="47">
+      <c r="M20" s="32">
         <v>4.0294606718451698E-2</v>
       </c>
-      <c r="N20" s="48">
+      <c r="N20" s="33">
         <v>4.1963339851818701E-2</v>
       </c>
     </row>
@@ -2379,18 +2363,18 @@
       <c r="G21" s="9">
         <v>4.7856639655370002E-4</v>
       </c>
-      <c r="I21" s="45"/>
-      <c r="J21" s="33"/>
-      <c r="K21" s="36" t="s">
+      <c r="I21" s="43"/>
+      <c r="J21" s="23"/>
+      <c r="K21" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="L21" s="36" t="s">
+      <c r="L21" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="M21" s="36" t="s">
+      <c r="M21" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="N21" s="49" t="s">
+      <c r="N21" s="34" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2416,20 +2400,20 @@
       <c r="G22" s="9">
         <v>7.9506872459265999E-3</v>
       </c>
-      <c r="I22" s="45"/>
-      <c r="J22" s="34" t="s">
-        <v>9</v>
-      </c>
-      <c r="K22" s="47">
+      <c r="I22" s="43"/>
+      <c r="J22" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="K22" s="32">
         <v>2.7877782388477702E-2</v>
       </c>
-      <c r="L22" s="47">
+      <c r="L22" s="32">
         <v>4.1004853919924297E-2</v>
       </c>
-      <c r="M22" s="47">
+      <c r="M22" s="32">
         <v>3.8771239271089601E-2</v>
       </c>
-      <c r="N22" s="44">
+      <c r="N22" s="30">
         <v>2.6563546292623599E-2</v>
       </c>
     </row>
@@ -2455,18 +2439,18 @@
       <c r="G23" s="10">
         <v>0.12891208974354801</v>
       </c>
-      <c r="I23" s="50"/>
-      <c r="J23" s="35"/>
+      <c r="I23" s="44"/>
+      <c r="J23" s="25"/>
       <c r="K23" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="L23" s="37" t="s">
+      <c r="L23" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="M23" s="37" t="s">
+      <c r="M23" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="N23" s="53" t="s">
+      <c r="N23" s="36" t="s">
         <v>35</v>
       </c>
     </row>
@@ -2492,22 +2476,22 @@
       <c r="G24" s="10">
         <v>8.7196464352812999E-3</v>
       </c>
-      <c r="I24" s="52">
+      <c r="I24" s="42">
         <v>12</v>
       </c>
-      <c r="J24" s="32" t="s">
+      <c r="J24" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="K24" s="21">
+      <c r="K24" s="14">
         <v>-6.2206069450507998E-3</v>
       </c>
-      <c r="L24" s="21">
+      <c r="L24" s="14">
         <v>-6.9457633388909999E-4</v>
       </c>
-      <c r="M24" s="21">
+      <c r="M24" s="14">
         <v>1.7274350360729E-2</v>
       </c>
-      <c r="N24" s="48">
+      <c r="N24" s="33">
         <v>4.7582304856785398E-2</v>
       </c>
     </row>
@@ -2533,18 +2517,18 @@
       <c r="G25" s="10">
         <v>0.208888402471089</v>
       </c>
-      <c r="I25" s="45"/>
-      <c r="J25" s="33"/>
-      <c r="K25" s="25" t="s">
+      <c r="I25" s="43"/>
+      <c r="J25" s="23"/>
+      <c r="K25" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="L25" s="25" t="s">
+      <c r="L25" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="M25" s="25" t="s">
+      <c r="M25" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="N25" s="54" t="s">
+      <c r="N25" s="37" t="s">
         <v>38</v>
       </c>
     </row>
@@ -2570,20 +2554,20 @@
       <c r="G26" s="9">
         <v>0.95805729432186704</v>
       </c>
-      <c r="I26" s="45"/>
-      <c r="J26" s="32" t="s">
+      <c r="I26" s="43"/>
+      <c r="J26" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="K26" s="21">
+      <c r="K26" s="14">
         <v>1.55610672921839E-2</v>
       </c>
-      <c r="L26" s="21">
+      <c r="L26" s="14">
         <v>2.14332070845108E-2</v>
       </c>
-      <c r="M26" s="21">
+      <c r="M26" s="14">
         <v>3.3700752615642197E-2</v>
       </c>
-      <c r="N26" s="48">
+      <c r="N26" s="33">
         <v>5.05347405509049E-2</v>
       </c>
     </row>
@@ -2609,18 +2593,18 @@
       <c r="G27" s="9">
         <v>1.6370331429953E-3</v>
       </c>
-      <c r="I27" s="45"/>
-      <c r="J27" s="33"/>
-      <c r="K27" s="25" t="s">
+      <c r="I27" s="43"/>
+      <c r="J27" s="23"/>
+      <c r="K27" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="L27" s="25" t="s">
+      <c r="L27" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="M27" s="25" t="s">
+      <c r="M27" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="N27" s="54" t="s">
+      <c r="N27" s="37" t="s">
         <v>41</v>
       </c>
     </row>
@@ -2646,20 +2630,20 @@
       <c r="G28" s="9">
         <v>4.6583346619845003E-3</v>
       </c>
-      <c r="I28" s="45"/>
-      <c r="J28" s="34" t="s">
-        <v>9</v>
-      </c>
-      <c r="K28" s="47">
+      <c r="I28" s="43"/>
+      <c r="J28" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="K28" s="32">
         <v>2.1781674237234702E-2</v>
       </c>
-      <c r="L28" s="60">
+      <c r="L28" s="14">
         <v>2.21277834183999E-2</v>
       </c>
-      <c r="M28" s="60">
+      <c r="M28" s="14">
         <v>1.6426402254913201E-2</v>
       </c>
-      <c r="N28" s="44">
+      <c r="N28" s="30">
         <v>2.9524356941194999E-3</v>
       </c>
     </row>
@@ -2685,18 +2669,18 @@
       <c r="G29" s="10">
         <v>0.96471301456515401</v>
       </c>
-      <c r="I29" s="55"/>
-      <c r="J29" s="56"/>
-      <c r="K29" s="57" t="s">
+      <c r="I29" s="45"/>
+      <c r="J29" s="38"/>
+      <c r="K29" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="L29" s="58" t="s">
+      <c r="L29" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="M29" s="58" t="s">
+      <c r="M29" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="N29" s="59" t="s">
+      <c r="N29" s="41" t="s">
         <v>44</v>
       </c>
     </row>
@@ -2830,10 +2814,10 @@
       <c r="G34" s="9">
         <v>1.4720291072391501E-2</v>
       </c>
-      <c r="K34" s="20"/>
-      <c r="L34" s="21"/>
-      <c r="M34" s="21"/>
-      <c r="N34" s="21"/>
+      <c r="K34" s="17"/>
+      <c r="L34" s="14"/>
+      <c r="M34" s="14"/>
+      <c r="N34" s="14"/>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
@@ -2857,10 +2841,10 @@
       <c r="G35" s="10">
         <v>0.43332043259999797</v>
       </c>
-      <c r="K35" s="22"/>
-      <c r="L35" s="23"/>
-      <c r="M35" s="23"/>
-      <c r="N35" s="23"/>
+      <c r="K35" s="18"/>
+      <c r="L35" s="16"/>
+      <c r="M35" s="16"/>
+      <c r="N35" s="16"/>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="7">
@@ -2884,10 +2868,10 @@
       <c r="G36" s="10">
         <v>5.0155542116857701E-2</v>
       </c>
-      <c r="K36" s="21"/>
-      <c r="L36" s="21"/>
-      <c r="M36" s="21"/>
-      <c r="N36" s="21"/>
+      <c r="K36" s="14"/>
+      <c r="L36" s="14"/>
+      <c r="M36" s="14"/>
+      <c r="N36" s="14"/>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
@@ -2911,10 +2895,10 @@
       <c r="G37" s="10">
         <v>0.17395011282650499</v>
       </c>
-      <c r="K37" s="23"/>
-      <c r="L37" s="23"/>
-      <c r="M37" s="23"/>
-      <c r="N37" s="23"/>
+      <c r="K37" s="16"/>
+      <c r="L37" s="16"/>
+      <c r="M37" s="16"/>
+      <c r="N37" s="16"/>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="6">
@@ -2938,10 +2922,10 @@
       <c r="G38" s="9">
         <v>0.59321870892864503</v>
       </c>
-      <c r="K38" s="21"/>
-      <c r="L38" s="21"/>
-      <c r="M38" s="21"/>
-      <c r="N38" s="21"/>
+      <c r="K38" s="14"/>
+      <c r="L38" s="14"/>
+      <c r="M38" s="14"/>
+      <c r="N38" s="14"/>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="6">
@@ -2965,10 +2949,10 @@
       <c r="G39" s="9">
         <v>7.9953173706632505E-2</v>
       </c>
-      <c r="K39" s="23"/>
-      <c r="L39" s="23"/>
-      <c r="M39" s="23"/>
-      <c r="N39" s="23"/>
+      <c r="K39" s="16"/>
+      <c r="L39" s="16"/>
+      <c r="M39" s="16"/>
+      <c r="N39" s="16"/>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
@@ -2992,10 +2976,10 @@
       <c r="G40" s="9">
         <v>3.1175742226854802E-2</v>
       </c>
-      <c r="K40" s="21"/>
-      <c r="L40" s="21"/>
-      <c r="M40" s="21"/>
-      <c r="N40" s="21"/>
+      <c r="K40" s="14"/>
+      <c r="L40" s="14"/>
+      <c r="M40" s="14"/>
+      <c r="N40" s="14"/>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" s="7">
@@ -3019,10 +3003,10 @@
       <c r="G41" s="10">
         <v>0.96266821624608201</v>
       </c>
-      <c r="K41" s="23"/>
-      <c r="L41" s="23"/>
-      <c r="M41" s="23"/>
-      <c r="N41" s="23"/>
+      <c r="K41" s="16"/>
+      <c r="L41" s="16"/>
+      <c r="M41" s="16"/>
+      <c r="N41" s="16"/>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
@@ -3046,10 +3030,10 @@
       <c r="G42" s="10">
         <v>0.11567711128970599</v>
       </c>
-      <c r="K42" s="20"/>
-      <c r="L42" s="21"/>
-      <c r="M42" s="21"/>
-      <c r="N42" s="21"/>
+      <c r="K42" s="17"/>
+      <c r="L42" s="14"/>
+      <c r="M42" s="14"/>
+      <c r="N42" s="14"/>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" s="7">
@@ -3073,10 +3057,10 @@
       <c r="G43" s="10">
         <v>0.119860281551464</v>
       </c>
-      <c r="K43" s="22"/>
-      <c r="L43" s="23"/>
-      <c r="M43" s="23"/>
-      <c r="N43" s="23"/>
+      <c r="K43" s="18"/>
+      <c r="L43" s="16"/>
+      <c r="M43" s="16"/>
+      <c r="N43" s="16"/>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="6">
@@ -3100,10 +3084,10 @@
       <c r="G44" s="9">
         <v>0.335830909036957</v>
       </c>
-      <c r="K44" s="20"/>
-      <c r="L44" s="21"/>
-      <c r="M44" s="21"/>
-      <c r="N44" s="21"/>
+      <c r="K44" s="17"/>
+      <c r="L44" s="14"/>
+      <c r="M44" s="14"/>
+      <c r="N44" s="14"/>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="6">
@@ -3127,10 +3111,10 @@
       <c r="G45" s="9">
         <v>5.8902534117065301E-2</v>
       </c>
-      <c r="K45" s="22"/>
-      <c r="L45" s="23"/>
-      <c r="M45" s="23"/>
-      <c r="N45" s="23"/>
+      <c r="K45" s="18"/>
+      <c r="L45" s="16"/>
+      <c r="M45" s="16"/>
+      <c r="N45" s="16"/>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="6">
@@ -3154,10 +3138,10 @@
       <c r="G46" s="9">
         <v>0.35402843630614</v>
       </c>
-      <c r="K46" s="20"/>
-      <c r="L46" s="21"/>
-      <c r="M46" s="21"/>
-      <c r="N46" s="21"/>
+      <c r="K46" s="17"/>
+      <c r="L46" s="14"/>
+      <c r="M46" s="14"/>
+      <c r="N46" s="14"/>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
@@ -3181,10 +3165,10 @@
       <c r="G47" s="10">
         <v>3.5588701036567499E-2</v>
       </c>
-      <c r="K47" s="22"/>
-      <c r="L47" s="23"/>
-      <c r="M47" s="23"/>
-      <c r="N47" s="23"/>
+      <c r="K47" s="18"/>
+      <c r="L47" s="16"/>
+      <c r="M47" s="16"/>
+      <c r="N47" s="16"/>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="7">
@@ -3208,10 +3192,10 @@
       <c r="G48" s="10">
         <v>2.6971310954366098E-2</v>
       </c>
-      <c r="K48" s="21"/>
-      <c r="L48" s="21"/>
-      <c r="M48" s="21"/>
-      <c r="N48" s="21"/>
+      <c r="K48" s="14"/>
+      <c r="L48" s="14"/>
+      <c r="M48" s="14"/>
+      <c r="N48" s="14"/>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
@@ -3235,82 +3219,70 @@
       <c r="G49" s="10">
         <v>0.90054726036784105</v>
       </c>
-      <c r="K49" s="23"/>
-      <c r="L49" s="23"/>
-      <c r="M49" s="23"/>
-      <c r="N49" s="23"/>
+      <c r="K49" s="16"/>
+      <c r="L49" s="16"/>
+      <c r="M49" s="16"/>
+      <c r="N49" s="16"/>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K50" s="21"/>
-      <c r="L50" s="21"/>
-      <c r="M50" s="21"/>
-      <c r="N50" s="21"/>
+      <c r="K50" s="14"/>
+      <c r="L50" s="14"/>
+      <c r="M50" s="14"/>
+      <c r="N50" s="14"/>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K51" s="23"/>
-      <c r="L51" s="23"/>
-      <c r="M51" s="23"/>
-      <c r="N51" s="23"/>
+      <c r="K51" s="16"/>
+      <c r="L51" s="16"/>
+      <c r="M51" s="16"/>
+      <c r="N51" s="16"/>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K52" s="21"/>
-      <c r="L52" s="21"/>
-      <c r="M52" s="21"/>
-      <c r="N52" s="21"/>
+      <c r="K52" s="14"/>
+      <c r="L52" s="14"/>
+      <c r="M52" s="14"/>
+      <c r="N52" s="14"/>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K53" s="23"/>
-      <c r="L53" s="23"/>
-      <c r="M53" s="23"/>
-      <c r="N53" s="23"/>
+      <c r="K53" s="16"/>
+      <c r="L53" s="16"/>
+      <c r="M53" s="16"/>
+      <c r="N53" s="16"/>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K54" s="21"/>
-      <c r="L54" s="21"/>
-      <c r="M54" s="21"/>
-      <c r="N54" s="21"/>
+      <c r="K54" s="14"/>
+      <c r="L54" s="14"/>
+      <c r="M54" s="14"/>
+      <c r="N54" s="14"/>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K55" s="23"/>
-      <c r="L55" s="23"/>
-      <c r="M55" s="23"/>
-      <c r="N55" s="23"/>
+      <c r="K55" s="16"/>
+      <c r="L55" s="16"/>
+      <c r="M55" s="16"/>
+      <c r="N55" s="16"/>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K56" s="21"/>
-      <c r="L56" s="21"/>
-      <c r="M56" s="21"/>
-      <c r="N56" s="21"/>
+      <c r="K56" s="14"/>
+      <c r="L56" s="14"/>
+      <c r="M56" s="14"/>
+      <c r="N56" s="14"/>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K57" s="23"/>
-      <c r="L57" s="23"/>
-      <c r="M57" s="23"/>
-      <c r="N57" s="23"/>
+      <c r="K57" s="16"/>
+      <c r="L57" s="16"/>
+      <c r="M57" s="16"/>
+      <c r="N57" s="16"/>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K58" s="21"/>
-      <c r="L58" s="21"/>
-      <c r="M58" s="21"/>
-      <c r="N58" s="21"/>
+      <c r="K58" s="14"/>
+      <c r="L58" s="14"/>
+      <c r="M58" s="14"/>
+      <c r="N58" s="14"/>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K59" s="23"/>
-      <c r="L59" s="23"/>
-      <c r="M59" s="23"/>
-      <c r="N59" s="23"/>
-    </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K60" s="24"/>
-      <c r="L60" s="24"/>
-      <c r="M60" s="24"/>
-      <c r="N60" s="24"/>
-    </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="K61" s="24"/>
-      <c r="L61" s="24"/>
-      <c r="M61" s="24"/>
-      <c r="N61" s="24"/>
+      <c r="K59" s="16"/>
+      <c r="L59" s="16"/>
+      <c r="M59" s="16"/>
+      <c r="N59" s="16"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G49" xr:uid="{828DFD01-9D50-4EA6-A7DD-A0B766D34BA5}">
@@ -3345,4 +3317,24 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60641E96-17E1-4C28-95A7-3B3EADA10A6C}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <phoneticPr fontId="19" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BA12766-CA57-4195-AB5D-D953190D2612}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <phoneticPr fontId="19" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>